<commit_message>
doc: actualizacion informacion de redes y comandos nuevos, falta organizar los coandos
</commit_message>
<xml_diff>
--- a/4_excel/1_subneting.xlsx
+++ b/4_excel/1_subneting.xlsx
@@ -7,7 +7,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Administrator\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A7369E48-04C6-47D4-A5EC-EB4FA88322F7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B8D0710A-1030-4E85-8F56-B54F4C072B31}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}" activeTab="0"/>
   </bookViews>
@@ -142,14 +142,14 @@
     </font>
     <font>
       <name val="Arial"/>
-      <sz val="11.00"/>
-      <b/>
+      <sz val="15.00"/>
       <color rgb="FF000000"/>
       <family val="2"/>
     </font>
     <font>
       <name val="Arial"/>
-      <sz val="15.00"/>
+      <sz val="11.00"/>
+      <b/>
       <color rgb="FF000000"/>
       <family val="2"/>
     </font>
@@ -169,13 +169,13 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFC000"/>
+        <fgColor rgb="FFE97132"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF0F9ED5"/>
+        <fgColor rgb="FFD86ECC"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -199,13 +199,13 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFE97132"/>
+        <fgColor rgb="FF0F9ED5"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFD86ECC"/>
+        <fgColor rgb="FFFFC000"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -225,6 +225,47 @@
       <diagonal/>
     </border>
     <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
       <left/>
       <right style="thin">
         <color rgb="FF000000"/>
@@ -256,9 +297,7 @@
       <left style="thin">
         <color rgb="FF000000"/>
       </left>
-      <right style="thin">
-        <color rgb="FF000000"/>
-      </right>
+      <right/>
       <top style="thin">
         <color rgb="FF000000"/>
       </top>
@@ -283,6 +322,36 @@
       <diagonal/>
     </border>
     <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
       <left/>
       <right style="thin">
         <color rgb="FF000000"/>
@@ -309,17 +378,6 @@
       <diagonal/>
     </border>
     <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
       <left style="thin">
         <color rgb="FF000000"/>
       </left>
@@ -341,64 +399,6 @@
       <right style="thin">
         <color rgb="FF000000"/>
       </right>
-      <top style="thin">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF000000"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF000000"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF000000"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF000000"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF000000"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF000000"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF000000"/>
-      </left>
-      <right/>
       <top style="thin">
         <color rgb="FF000000"/>
       </top>
@@ -413,86 +413,86 @@
     <xf fontId="1" applyFont="1" fillId="2" applyFill="1" borderId="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf fontId="1" applyFont="1" fillId="3" applyFill="1" borderId="2" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf fontId="1" applyFont="1" borderId="3" applyBorder="1"/>
-    <xf fontId="1" applyFont="1" borderId="4" applyBorder="1" applyAlignment="1">
+    <xf fontId="2" applyFont="1" fillId="3" applyFill="1" borderId="2" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" horizontal="center"/>
     </xf>
+    <xf fontId="1" applyFont="1" fillId="4" applyFill="1" borderId="3" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf fontId="1" applyFont="1" fillId="5" applyFill="1" borderId="4" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf fontId="1" applyFont="1" borderId="5" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" horizontal="center"/>
+    </xf>
+    <xf fontId="1" applyFont="1" fillId="6" applyFill="1" borderId="6" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf fontId="3" applyFont="1" borderId="7" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" horizontal="center" wrapText="1"/>
+    </xf>
+    <xf fontId="1" applyFont="1" borderId="8" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf fontId="1" applyFont="1" fillId="7" applyFill="1" borderId="9" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf fontId="1" applyFont="1"/>
-    <xf fontId="1" applyFont="1" fillId="4" applyFill="1" borderId="5" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf fontId="1" applyFont="1" fillId="5" applyFill="1" borderId="6" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf fontId="1" applyFont="1" fillId="6" applyFill="1" borderId="7" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf fontId="1" applyFont="1" fillId="7" applyFill="1" borderId="8" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf fontId="2" applyFont="1" borderId="9" applyBorder="1" applyAlignment="1">
+    <xf fontId="1" applyFont="1" fillId="8" applyFill="1" borderId="10" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf fontId="2" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf fontId="1" applyFont="1" fillId="9" applyFill="1" borderId="11" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf fontId="1" applyFont="1" borderId="12" applyBorder="1"/>
+    <xf fontId="4" applyFont="1" borderId="13" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" horizontal="center" wrapText="1"/>
-    </xf>
-    <xf fontId="3" applyFont="1" fillId="8" applyFill="1" borderId="10" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" horizontal="center"/>
-    </xf>
-    <xf fontId="3" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf fontId="1" applyFont="1" borderId="11" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf fontId="4" applyFont="1" borderId="12" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" horizontal="center" wrapText="1"/>
-    </xf>
-    <xf fontId="1" applyFont="1" fillId="9" applyFill="1" borderId="13" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
   </cellStyleXfs>
   <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf xfId="7" quotePrefix="0" pivotButton="0" fontId="1" applyFont="1" fillId="5" applyFill="1" borderId="6" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf xfId="8" quotePrefix="0" pivotButton="0" fontId="1" applyFont="1" fillId="6" applyFill="1" borderId="7" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf xfId="6" quotePrefix="0" pivotButton="0" fontId="1" applyFont="1" fillId="4" applyFill="1" borderId="5" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf xfId="15" quotePrefix="0" pivotButton="0" fontId="1" applyFont="1" fillId="9" applyFill="1" borderId="13" applyBorder="1" applyAlignment="1">
+    <xf xfId="6" quotePrefix="0" pivotButton="0" fontId="1" applyFont="1" fillId="6" applyFill="1" borderId="6" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf xfId="3" quotePrefix="0" pivotButton="0" fontId="1" applyFont="1" fillId="4" applyFill="1" borderId="3" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf xfId="4" quotePrefix="0" pivotButton="0" fontId="1" applyFont="1" fillId="5" applyFill="1" borderId="4" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf xfId="13" quotePrefix="0" pivotButton="0" fontId="1" applyFont="1" fillId="9" applyFill="1" borderId="11" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf xfId="11" quotePrefix="0" pivotButton="0" fontId="1" applyFont="1" fillId="8" applyFill="1" borderId="10" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf xfId="1" quotePrefix="0" pivotButton="0" fontId="1" applyFont="1" fillId="2" applyFill="1" borderId="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf xfId="9" quotePrefix="0" pivotButton="0" fontId="1" applyFont="1" fillId="7" applyFill="1" borderId="8" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf xfId="13" quotePrefix="0" pivotButton="0" fontId="1" applyFont="1" borderId="11" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf xfId="4" quotePrefix="0" pivotButton="0" fontId="1" applyFont="1" borderId="4" applyBorder="1" applyAlignment="1">
+    <xf xfId="8" quotePrefix="0" pivotButton="0" fontId="1" applyFont="1" borderId="8" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf xfId="5" quotePrefix="0" pivotButton="0" fontId="1" applyFont="1" borderId="5" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" horizontal="center"/>
     </xf>
-    <xf xfId="3" quotePrefix="0" pivotButton="0" fontId="1" applyFont="1" borderId="3" applyBorder="1"/>
-    <xf xfId="2" quotePrefix="0" pivotButton="0" fontId="1" applyFont="1" fillId="3" applyFill="1" borderId="2" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf xfId="5" quotePrefix="0" pivotButton="0" fontId="1" applyFont="1"/>
-    <xf xfId="11" quotePrefix="0" pivotButton="0" fontId="3" applyFont="1" fillId="8" applyFill="1" borderId="10" applyBorder="1" applyAlignment="1">
+    <xf xfId="14" quotePrefix="0" pivotButton="0" fontId="1" applyFont="1" borderId="12" applyBorder="1"/>
+    <xf xfId="9" quotePrefix="0" pivotButton="0" fontId="1" applyFont="1" fillId="7" applyFill="1" borderId="9" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf xfId="10" quotePrefix="0" pivotButton="0" fontId="1" applyFont="1"/>
+    <xf xfId="2" quotePrefix="0" pivotButton="0" fontId="2" applyFont="1" fillId="3" applyFill="1" borderId="2" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" horizontal="center"/>
     </xf>
-    <xf xfId="10" quotePrefix="0" pivotButton="0" fontId="2" applyFont="1" borderId="9" applyBorder="1" applyAlignment="1">
+    <xf xfId="7" quotePrefix="0" pivotButton="0" fontId="3" applyFont="1" borderId="7" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" horizontal="center" wrapText="1"/>
     </xf>
-    <xf xfId="14" quotePrefix="0" pivotButton="0" fontId="4" applyFont="1" borderId="12" applyBorder="1" applyAlignment="1">
+    <xf xfId="15" quotePrefix="0" pivotButton="0" fontId="4" applyFont="1" borderId="13" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" horizontal="center" wrapText="1"/>
     </xf>
-    <xf xfId="12" quotePrefix="0" pivotButton="0" fontId="3" applyFont="1" applyAlignment="1">
+    <xf xfId="12" quotePrefix="0" pivotButton="0" fontId="2" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -787,7 +787,7 @@
     <col min="15" max="15" width="16.44" customWidth="1" hidden="0"/>
     <col min="16" max="16" width="19.99" customWidth="1" hidden="0"/>
     <col min="17" max="17" width="19.62" customWidth="1" hidden="0"/>
-    <col min="18" max="18" width="17.17" customWidth="1" hidden="0"/>
+    <col min="18" max="18" width="18.40" customWidth="1" hidden="0"/>
     <col min="19" max="19" width="20.11" customWidth="1" hidden="0"/>
   </cols>
   <sheetData>
@@ -840,7 +840,7 @@
         <v>0</v>
       </c>
       <c r="J2" s="7">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="K2" s="9" t="s">
         <v>3</v>

</xml_diff>